<commit_message>
Major updates to DOF importing script, included data visualization code for both ACS and DOF
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/BLS/config/BLS_State and Area Employment_Series ID Codes.xlsx
+++ b/Indicator_Gen/Python Code/BLS/config/BLS_State and Area Employment_Series ID Codes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sacog.sharepoint.com/sites/RegionalMonitoringandReporting/Shared Documents/Process Revamp/Task 9. Collect new data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{D11369E1-5776-4A57-BFA2-F789D30C5E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0331B726-895D-47CF-B0B4-0580987959CF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A8FD21-8E0A-4BB8-8EC8-71BA39C001B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -2638,7 +2638,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2668,12 +2668,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2729,7 +2723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2743,7 +2737,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7128,7 +7121,7 @@
       <c r="A319" t="s">
         <v>319</v>
       </c>
-      <c r="B319" s="7" t="s">
+      <c r="B319" t="s">
         <v>659</v>
       </c>
       <c r="C319" t="s">
@@ -7181,7 +7174,7 @@
       <c r="A323" t="s">
         <v>323</v>
       </c>
-      <c r="B323" s="7" t="s">
+      <c r="B323" t="s">
         <v>663</v>
       </c>
       <c r="C323" t="s">
@@ -7886,15 +7879,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -8123,15 +8107,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF250B34-2756-44A2-A030-8FEBB211D63C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8148,4 +8133,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Included state looping on tracts/county pulls in acs query script, updated BLS query scripts, started creating mapping from PUMA to county to MSA
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/BLS/config/BLS_State and Area Employment_Series ID Codes.xlsx
+++ b/Indicator_Gen/Python Code/BLS/config/BLS_State and Area Employment_Series ID Codes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A8FD21-8E0A-4BB8-8EC8-71BA39C001B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27457B48-0650-405B-8F2D-5424527FAE0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="835">
   <si>
     <t>industry_code</t>
   </si>
@@ -2343,12 +2343,6 @@
     <t>sp_folder</t>
   </si>
   <si>
-    <t>Themes</t>
-  </si>
-  <si>
-    <t>SharePoint Paths</t>
-  </si>
-  <si>
     <t>12420</t>
   </si>
   <si>
@@ -2358,12 +2352,6 @@
     <t>Vibrant and Inclusive Places</t>
   </si>
   <si>
-    <t>Economy\\Income</t>
-  </si>
-  <si>
-    <t>People and Community\\Pop and Demographics</t>
-  </si>
-  <si>
     <t>16740</t>
   </si>
   <si>
@@ -2379,18 +2367,12 @@
     <t>Cincinnati, OH-KY-IN Metro Area</t>
   </si>
   <si>
-    <t>Economy\\Education</t>
-  </si>
-  <si>
     <t>17460</t>
   </si>
   <si>
     <t>Cleveland-Elyria, OH Metro Area</t>
   </si>
   <si>
-    <t>People and Community\\Broadband</t>
-  </si>
-  <si>
     <t>18140</t>
   </si>
   <si>
@@ -2403,19 +2385,10 @@
     <t>Detroit-Warren-Dearborn, MI Metro Area</t>
   </si>
   <si>
-    <t>Next Gen of Mobility Solutions</t>
-  </si>
-  <si>
-    <t>Travel modes</t>
-  </si>
-  <si>
     <t>26900</t>
   </si>
   <si>
     <t>Indianapolis-Carmel-Anderson, IN Metro Area</t>
-  </si>
-  <si>
-    <t>People and Community\\Healthy Places</t>
   </si>
   <si>
     <t>28140</t>
@@ -3126,66 +3099,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>812</v>
+        <v>803</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>814</v>
+        <v>805</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>813</v>
+        <v>804</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>808</v>
+        <v>799</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>817</v>
+        <v>808</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>818</v>
+        <v>809</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="B10" t="s">
-        <v>819</v>
+        <v>810</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="B11" t="s">
-        <v>821</v>
+        <v>812</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>822</v>
+        <v>813</v>
       </c>
       <c r="B12" t="s">
-        <v>824</v>
+        <v>815</v>
       </c>
     </row>
   </sheetData>
@@ -3232,252 +3205,206 @@
       <c r="G1" s="4" t="s">
         <v>746</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>747</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>748</v>
-      </c>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C2" t="s">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="D2">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="E2">
         <v>2023</v>
       </c>
       <c r="F2" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="G2" t="s">
-        <v>756</v>
-      </c>
-      <c r="J2" t="s">
-        <v>751</v>
-      </c>
-      <c r="K2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="B3" t="s">
-        <v>755</v>
-      </c>
-      <c r="J3" t="s">
         <v>751</v>
-      </c>
-      <c r="K3" t="s">
-        <v>756</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="B4" t="s">
-        <v>758</v>
-      </c>
-      <c r="J4" t="s">
-        <v>751</v>
-      </c>
-      <c r="K4" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="B5" t="s">
-        <v>761</v>
-      </c>
-      <c r="J5" t="s">
-        <v>751</v>
-      </c>
-      <c r="K5" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="B6" t="s">
-        <v>764</v>
-      </c>
-      <c r="J6" t="s">
-        <v>751</v>
-      </c>
-      <c r="K6" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="B7" t="s">
-        <v>766</v>
-      </c>
-      <c r="J7" t="s">
-        <v>767</v>
-      </c>
-      <c r="K7" t="s">
-        <v>768</v>
+        <v>760</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>769</v>
+        <v>761</v>
       </c>
       <c r="B8" t="s">
-        <v>770</v>
-      </c>
-      <c r="J8" t="s">
-        <v>751</v>
-      </c>
-      <c r="K8" t="s">
-        <v>771</v>
+        <v>762</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>772</v>
+        <v>763</v>
       </c>
       <c r="B9" t="s">
-        <v>773</v>
+        <v>764</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>774</v>
+        <v>765</v>
       </c>
       <c r="B10" t="s">
-        <v>775</v>
+        <v>766</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>776</v>
+        <v>767</v>
       </c>
       <c r="B11" t="s">
-        <v>777</v>
+        <v>768</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>778</v>
+        <v>769</v>
       </c>
       <c r="B12" t="s">
-        <v>779</v>
+        <v>770</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>780</v>
+        <v>771</v>
       </c>
       <c r="B13" t="s">
-        <v>781</v>
+        <v>772</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>782</v>
+        <v>773</v>
       </c>
       <c r="B14" t="s">
-        <v>783</v>
+        <v>774</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>784</v>
+        <v>775</v>
       </c>
       <c r="B15" t="s">
-        <v>785</v>
+        <v>776</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>786</v>
+        <v>777</v>
       </c>
       <c r="B16" t="s">
-        <v>787</v>
+        <v>778</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>788</v>
+        <v>779</v>
       </c>
       <c r="B17" t="s">
-        <v>789</v>
+        <v>780</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>790</v>
+        <v>781</v>
       </c>
       <c r="B18" t="s">
-        <v>791</v>
+        <v>782</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>792</v>
+        <v>783</v>
       </c>
       <c r="B19" t="s">
-        <v>793</v>
+        <v>784</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>794</v>
+        <v>785</v>
       </c>
       <c r="B20" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>796</v>
+        <v>787</v>
       </c>
       <c r="B21" t="s">
-        <v>797</v>
+        <v>788</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>798</v>
+        <v>789</v>
       </c>
       <c r="B22" t="s">
-        <v>799</v>
+        <v>790</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>800</v>
+        <v>791</v>
       </c>
       <c r="B23" t="s">
-        <v>801</v>
+        <v>792</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>802</v>
+        <v>793</v>
       </c>
       <c r="B24" t="s">
-        <v>803</v>
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -3507,7 +3434,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>823</v>
+        <v>814</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>736</v>
@@ -3530,13 +3457,13 @@
         <v>342</v>
       </c>
       <c r="C2" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="E2" t="s">
         <v>739</v>
       </c>
       <c r="G2" t="s">
-        <v>808</v>
+        <v>799</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3547,13 +3474,13 @@
         <v>343</v>
       </c>
       <c r="C3" t="s">
-        <v>836</v>
+        <v>827</v>
       </c>
       <c r="E3" t="s">
         <v>739</v>
       </c>
       <c r="G3" t="s">
-        <v>807</v>
+        <v>798</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -3564,7 +3491,7 @@
         <v>344</v>
       </c>
       <c r="C4" t="s">
-        <v>822</v>
+        <v>813</v>
       </c>
       <c r="E4" t="s">
         <v>739</v>
@@ -3578,7 +3505,7 @@
         <v>345</v>
       </c>
       <c r="C5" t="s">
-        <v>822</v>
+        <v>813</v>
       </c>
       <c r="E5" t="s">
         <v>739</v>
@@ -3603,7 +3530,7 @@
         <v>347</v>
       </c>
       <c r="C7" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D7" t="s">
         <v>347</v>
@@ -3730,7 +3657,7 @@
         <v>358</v>
       </c>
       <c r="C18" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D18" t="s">
         <v>358</v>
@@ -3890,7 +3817,7 @@
         <v>372</v>
       </c>
       <c r="C32" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D32" t="s">
         <v>372</v>
@@ -4765,10 +4692,10 @@
         <v>451</v>
       </c>
       <c r="C111" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D111" t="s">
-        <v>826</v>
+        <v>817</v>
       </c>
       <c r="E111" t="s">
         <v>737</v>
@@ -4958,10 +4885,10 @@
         <v>468</v>
       </c>
       <c r="C128" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D128" t="s">
-        <v>827</v>
+        <v>818</v>
       </c>
       <c r="E128" t="s">
         <v>737</v>
@@ -5294,10 +5221,10 @@
         <v>498</v>
       </c>
       <c r="C158" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D158" t="s">
-        <v>826</v>
+        <v>817</v>
       </c>
       <c r="E158" t="s">
         <v>737</v>
@@ -5553,10 +5480,10 @@
         <v>521</v>
       </c>
       <c r="C181" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D181" t="s">
-        <v>828</v>
+        <v>819</v>
       </c>
       <c r="E181" t="s">
         <v>737</v>
@@ -5724,10 +5651,10 @@
         <v>536</v>
       </c>
       <c r="C196" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D196" t="s">
-        <v>828</v>
+        <v>819</v>
       </c>
       <c r="E196" t="s">
         <v>737</v>
@@ -6027,7 +5954,7 @@
         <v>563</v>
       </c>
       <c r="C223" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D223" t="s">
         <v>563</v>
@@ -6330,16 +6257,16 @@
         <v>590</v>
       </c>
       <c r="C250" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D250" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="E250" t="s">
         <v>737</v>
       </c>
       <c r="F250" t="s">
-        <v>811</v>
+        <v>802</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.35">
@@ -6350,7 +6277,7 @@
         <v>591</v>
       </c>
       <c r="E251" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.35">
@@ -6361,7 +6288,7 @@
         <v>592</v>
       </c>
       <c r="E252" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.35">
@@ -6372,7 +6299,7 @@
         <v>593</v>
       </c>
       <c r="E253" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.35">
@@ -6383,7 +6310,7 @@
         <v>594</v>
       </c>
       <c r="E254" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.35">
@@ -6394,10 +6321,10 @@
         <v>595</v>
       </c>
       <c r="C255" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D255" t="s">
-        <v>830</v>
+        <v>821</v>
       </c>
       <c r="E255" t="s">
         <v>737</v>
@@ -6664,10 +6591,10 @@
         <v>619</v>
       </c>
       <c r="C279" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D279" t="s">
-        <v>831</v>
+        <v>822</v>
       </c>
       <c r="E279" t="s">
         <v>737</v>
@@ -6934,7 +6861,7 @@
         <v>643</v>
       </c>
       <c r="C303" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D303" t="s">
         <v>643</v>
@@ -7105,7 +7032,7 @@
         <v>658</v>
       </c>
       <c r="C318" t="s">
-        <v>837</v>
+        <v>828</v>
       </c>
       <c r="D318" t="s">
         <v>658</v>
@@ -7114,7 +7041,7 @@
         <v>737</v>
       </c>
       <c r="F318" t="s">
-        <v>832</v>
+        <v>823</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.35">
@@ -7125,7 +7052,7 @@
         <v>659</v>
       </c>
       <c r="C319" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D319" t="s">
         <v>659</v>
@@ -7134,7 +7061,7 @@
         <v>737</v>
       </c>
       <c r="F319" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.35">
@@ -7178,16 +7105,16 @@
         <v>663</v>
       </c>
       <c r="C323" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D323" t="s">
-        <v>830</v>
+        <v>821</v>
       </c>
       <c r="E323" t="s">
         <v>737</v>
       </c>
       <c r="F323" s="6" t="s">
-        <v>841</v>
+        <v>832</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.35">
@@ -7253,16 +7180,16 @@
         <v>669</v>
       </c>
       <c r="C329" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D329" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="E329" t="s">
         <v>737</v>
       </c>
       <c r="F329" t="s">
-        <v>833</v>
+        <v>824</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.35">
@@ -7284,10 +7211,10 @@
         <v>671</v>
       </c>
       <c r="C331" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D331" t="s">
-        <v>830</v>
+        <v>821</v>
       </c>
       <c r="E331" t="s">
         <v>737</v>
@@ -7301,7 +7228,7 @@
         <v>672</v>
       </c>
       <c r="C332" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D332" t="s">
         <v>668</v>
@@ -7310,7 +7237,7 @@
         <v>737</v>
       </c>
       <c r="F332" t="s">
-        <v>842</v>
+        <v>833</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.35">
@@ -7343,16 +7270,16 @@
         <v>675</v>
       </c>
       <c r="C335" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D335" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="E335" t="s">
         <v>737</v>
       </c>
       <c r="F335" t="s">
-        <v>834</v>
+        <v>825</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.35">
@@ -7363,7 +7290,7 @@
         <v>676</v>
       </c>
       <c r="C336" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D336" t="s">
         <v>673</v>
@@ -7372,7 +7299,7 @@
         <v>737</v>
       </c>
       <c r="F336" t="s">
-        <v>843</v>
+        <v>834</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.35">
@@ -7383,16 +7310,16 @@
         <v>677</v>
       </c>
       <c r="C337" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D337" t="s">
-        <v>826</v>
+        <v>817</v>
       </c>
       <c r="E337" t="s">
         <v>737</v>
       </c>
       <c r="F337" t="s">
-        <v>835</v>
+        <v>826</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.35">
@@ -7403,16 +7330,16 @@
         <v>678</v>
       </c>
       <c r="C338" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="D338" t="s">
-        <v>830</v>
+        <v>821</v>
       </c>
       <c r="E338" t="s">
         <v>737</v>
       </c>
       <c r="F338" t="s">
-        <v>835</v>
+        <v>826</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.35">
@@ -7423,13 +7350,13 @@
         <v>679</v>
       </c>
       <c r="D339" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="E339" t="s">
-        <v>840</v>
+        <v>831</v>
       </c>
       <c r="F339" t="s">
-        <v>834</v>
+        <v>825</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.35">
@@ -7645,7 +7572,7 @@
         <v>708</v>
       </c>
       <c r="F20" t="s">
-        <v>809</v>
+        <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -7672,12 +7599,12 @@
         <v>658</v>
       </c>
       <c r="F23" t="s">
-        <v>810</v>
+        <v>801</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F24" t="s">
-        <v>811</v>
+        <v>802</v>
       </c>
     </row>
   </sheetData>
@@ -7728,7 +7655,7 @@
         <v>720</v>
       </c>
       <c r="C2" t="s">
-        <v>805</v>
+        <v>796</v>
       </c>
       <c r="D2" t="s">
         <v>737</v>
@@ -7737,7 +7664,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>825</v>
+        <v>816</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -7879,6 +7806,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -8107,16 +8043,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF250B34-2756-44A2-A030-8FEBB211D63C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8133,12 +8068,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>